<commit_message>
New Code: Excel data reader
</commit_message>
<xml_diff>
--- a/SeleniumFrameworkDesign/src/main/java/org/resources/TestData.xlsx
+++ b/SeleniumFrameworkDesign/src/main/java/org/resources/TestData.xlsx
@@ -3,14 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20361"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A03C00A-DC12-463E-8D54-01AD6C148CB3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{7B1AD50A-C020-49ED-B452-3ACDAD2F798E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14925" windowHeight="5985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="TestData" sheetId="1" r:id="rId1"/>
+    <sheet name="Testdata" sheetId="1" r:id="rId1"/>
+    <sheet name="Sample" sheetId="2" r:id="rId2"/>
+    <sheet name="Demo" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -461,4 +464,22 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A46565F9-41BF-441C-AB74-A48C23F24CB2}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97F9F1BB-C3A8-4C2A-B2E3-92AF4A57D530}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>